<commit_message>
fix: 5 troncales sin shapefile por ID distinto al archivo (Montanuelo-Gualanday y 4 mas)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Listado de Infraestructura para Cod Informes.xlsx
+++ b/Listado de Infraestructura para Cod Informes.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="10245" yWindow="0" windowWidth="10245" windowHeight="10920" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hoja1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Hoja1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hoja1'!$B$1:$C$285</definedName>
@@ -2818,7 +2818,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>R_MNT</t>
+          <t>T_MON_GUA</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">

</xml_diff>